<commit_message>
Add 48 listicle firms missed as full-service, including WebFX
Co-authored-by: abaszeinn-beep <abaszeinn-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/excel/Autommerce_Partners_Kuwait.xlsx
+++ b/data/excel/Autommerce_Partners_Kuwait.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Partners" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Partners'!$A$1:$D$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Partners'!$A$1:$D$74</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D71"/>
+  <dimension ref="A1:D74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1432,17 +1432,17 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Creativity Business Solutions</t>
+          <t>Walnut Software Solutions</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>https://creativity.com.kw</t>
+          <t>https://walnutit.com</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Ecommerce System Integration Companies</t>
+          <t>Ecommerce PIM / ERP / Inventory Management Consultants</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -1454,39 +1454,39 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Nizek</t>
+          <t>Plennix Technologies</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>https://nizek.com</t>
+          <t>https://plennix.com</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Ecommerce Technology &amp; Digital Transformation Firms</t>
+          <t>Ecommerce PIM / ERP / Inventory Management Consultants</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Autommerce OS</t>
+          <t>Both</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>TechGropse</t>
+          <t>Pro Comrades</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>https://techgropse.com</t>
+          <t>https://procomrades.com</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Fashion Ecommerce Technology Consultants</t>
+          <t>Ecommerce PIM / ERP / Inventory Management Consultants</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -1498,17 +1498,17 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Techfriar</t>
+          <t>Creativity Business Solutions</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>https://techfriar.com</t>
+          <t>https://creativity.com.kw</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Ecommerce Website Development Agencies</t>
+          <t>Ecommerce System Integration Companies</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -1520,12 +1520,12 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Eurisko</t>
+          <t>Nizek</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>https://eurisko.net</t>
+          <t>https://nizek.com</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -1535,85 +1535,85 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Autommerce OS</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>IIH Global</t>
+          <t>TechGropse</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>https://iihglobal.com</t>
+          <t>https://techgropse.com</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Ecommerce Website Development Agencies</t>
+          <t>Fashion Ecommerce Technology Consultants</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Autommerce OS</t>
+          <t>Both</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>DevelopmentNow</t>
+          <t>Techfriar</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>https://developmentnow.com</t>
+          <t>https://techfriar.com</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Ecommerce System Integration Companies</t>
+          <t>Ecommerce Website Development Agencies</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Autommerce OS</t>
+          <t>Both</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Tenet</t>
+          <t>Eurisko</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>https://wearetenet.com</t>
+          <t>https://eurisko.net</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Ecommerce CRO &amp; UX/UI Agencies</t>
+          <t>Ecommerce Technology &amp; Digital Transformation Firms</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Autommerce OS</t>
+          <t>Both</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Inchoo</t>
+          <t>IIH Global</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>https://inchoo.net</t>
+          <t>https://iihglobal.com</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -1623,46 +1623,46 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Autommerce OS</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Mulanen</t>
+          <t>DevelopmentNow</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>https://mulanen.com</t>
+          <t>https://developmentnow.com</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Fashion Ecommerce Digital Marketing Agencies</t>
+          <t>Ecommerce System Integration Companies</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Autommerce OS</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>OntargIT</t>
+          <t>Tenet</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>https://ontargit.com</t>
+          <t>https://wearetenet.com</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Ecommerce PIM / ERP / Inventory Management Consultants</t>
+          <t>Ecommerce CRO &amp; UX/UI Agencies</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -1674,17 +1674,17 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Codilar</t>
+          <t>Inchoo</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>https://codilar.com</t>
+          <t>https://inchoo.net</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Ecommerce PIM / ERP / Inventory Management Consultants</t>
+          <t>Ecommerce Website Development Agencies</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -1696,17 +1696,17 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>AGM Global Services</t>
+          <t>Mulanen</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>https://agmglobal.co</t>
+          <t>https://mulanen.com</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Ecommerce PIM / ERP / Inventory Management Consultants</t>
+          <t>Fashion Ecommerce Digital Marketing Agencies</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -1718,39 +1718,39 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Gravityer</t>
+          <t>OntargIT</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>https://gravityer.com</t>
+          <t>https://ontargit.com</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Fashion Ecommerce Personalization &amp; Customer Experience Agencies</t>
+          <t>Ecommerce PIM / ERP / Inventory Management Consultants</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Autommerce OS</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Odyssey</t>
+          <t>Codilar</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>https://odysseymedia.co</t>
+          <t>https://codilar.com</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Ecommerce Product Photography &amp; Creative Production Agencies</t>
+          <t>Ecommerce PIM / ERP / Inventory Management Consultants</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -1762,12 +1762,12 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Seventh Dimension</t>
+          <t>AGM Global Services</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>https://7d.com.kw</t>
+          <t>https://agmglobal.co</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -1777,85 +1777,85 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Autommerce OS</t>
+          <t>Both</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Sapours</t>
+          <t>Gravityer</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>https://sapours.com</t>
+          <t>https://gravityer.com</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Ecommerce System Integration Companies</t>
+          <t>Fashion Ecommerce Personalization &amp; Customer Experience Agencies</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Autommerce OS</t>
+          <t>Both</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Cybage</t>
+          <t>Odyssey</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>https://cybage.com</t>
+          <t>https://odysseymedia.co</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Ecommerce System Integration Companies</t>
+          <t>Ecommerce Product Photography &amp; Creative Production Agencies</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Autommerce OS</t>
+          <t>Both</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Synoptek</t>
+          <t>Seventh Dimension</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>https://synoptek.com</t>
+          <t>https://7d.com.kw</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Ecommerce System Integration Companies</t>
+          <t>Ecommerce PIM / ERP / Inventory Management Consultants</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Autommerce OS</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>DTC Infotech</t>
+          <t>Sapours</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>https://dtcinfotech.com</t>
+          <t>https://sapours.com</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -1872,100 +1872,100 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Cliqtechno</t>
+          <t>Cybage</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>https://cliqtechno.com</t>
+          <t>https://cybage.com</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Ecommerce Website Development Agencies</t>
+          <t>Ecommerce System Integration Companies</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Autommerce OS</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Webkul</t>
+          <t>Synoptek</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>https://webkul.com</t>
+          <t>https://synoptek.com</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Ecommerce Website Development Agencies</t>
+          <t>Ecommerce System Integration Companies</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Autommerce OS</t>
+          <t>Both</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Klay Create</t>
+          <t>DTC Infotech</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>https://klaycreate.com</t>
+          <t>https://dtcinfotech.com</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Ecommerce Website Development Agencies</t>
+          <t>Ecommerce System Integration Companies</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Autommerce OS</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>CentrixPlus</t>
+          <t>Cliqtechno</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>https://centrixplus.com</t>
+          <t>https://cliqtechno.com</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Ecommerce PIM / ERP / Inventory Management Consultants</t>
+          <t>Ecommerce Website Development Agencies</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Autommerce OS</t>
+          <t>Both</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Tarawud</t>
+          <t>Webkul</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>https://tarawud.com</t>
+          <t>https://webkul.com</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -1975,34 +1975,100 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Autommerce OS</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
+          <t>Klay Create</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>https://klaycreate.com</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Ecommerce Website Development Agencies</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>CentrixPlus</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>https://centrixplus.com</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Ecommerce PIM / ERP / Inventory Management Consultants</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Autommerce OS</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Tarawud</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>https://tarawud.com</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Ecommerce Website Development Agencies</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
           <t>Bazaar Studios</t>
         </is>
       </c>
-      <c r="B71" s="2" t="inlineStr">
+      <c r="B74" s="2" t="inlineStr">
         <is>
           <t>https://bazaarstudios.com</t>
         </is>
       </c>
-      <c r="C71" s="2" t="inlineStr">
+      <c r="C74" s="2" t="inlineStr">
         <is>
           <t>Ecommerce Product Photography &amp; Creative Production Agencies</t>
         </is>
       </c>
-      <c r="D71" s="2" t="inlineStr">
+      <c r="D74" s="2" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D71"/>
+  <autoFilter ref="A1:D74"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 26 partner rows supplied for Kuwait, Lebanon, Qatar, Saudi Arabia, UAE, and the US
Co-authored-by: abaszeinn-beep <abaszeinn-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/excel/Autommerce_Partners_Kuwait.xlsx
+++ b/data/excel/Autommerce_Partners_Kuwait.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Partners" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Partners'!$A$1:$D$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Partners'!$A$1:$D$78</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D74"/>
+  <dimension ref="A1:D78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2067,8 +2067,96 @@
         </is>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Digitize Growth</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>https://digitizegrowth.com</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Ecommerce Website Development Agencies</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>SellThru</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>https://sellthruagency.com</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Ecommerce Digital Marketing &amp; Performance Agencies</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>ARQQA</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>https://arqqa.net</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Fashion Ecommerce Digital Marketing Agencies</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Cyber Sphere Enterprise</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>https://csekw.com</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Ecommerce Website Development Agencies</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D74"/>
+  <autoFilter ref="A1:D78"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add outreach contacts and decision makers to the partner workbooks.
Each market file now has a Company details sheet and a Decision makers sheet. Contact fields are filled only where research has already been saved.

Co-authored-by: abaszeinn-beep <abaszeinn-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/excel/Autommerce_Partners_Kuwait.xlsx
+++ b/data/excel/Autommerce_Partners_Kuwait.xlsx
@@ -7,10 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Partners" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company details" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision makers" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Partners'!$A$1:$D$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Company details'!$A$1:$G$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Decision makers'!$A$1:$G$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,8 +30,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -60,10 +68,10 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -427,19 +435,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F4E79"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D78"/>
+  <dimension ref="A1:G78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="72" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Company Name</t>
@@ -458,6 +470,21 @@
       <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Product Fit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Emails</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
         </is>
       </c>
     </row>
@@ -482,6 +509,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -504,6 +534,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -526,6 +559,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -548,6 +584,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -570,6 +609,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -592,6 +634,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -614,6 +659,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -636,6 +684,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -658,6 +709,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -680,6 +734,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -702,6 +759,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -724,6 +784,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -746,6 +809,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -768,6 +834,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -790,6 +859,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -812,6 +884,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -834,6 +909,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -856,6 +934,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -878,6 +959,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -900,6 +984,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -922,6 +1009,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -944,6 +1034,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -966,6 +1059,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -988,6 +1084,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1010,6 +1109,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1032,6 +1134,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1054,6 +1159,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1076,6 +1184,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1098,6 +1209,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1120,6 +1234,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1142,6 +1259,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1164,6 +1284,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1186,6 +1309,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1208,6 +1334,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1230,6 +1359,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1252,6 +1384,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1274,6 +1409,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr"/>
+      <c r="G38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1296,6 +1434,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E39" s="2" t="inlineStr"/>
+      <c r="F39" s="2" t="inlineStr"/>
+      <c r="G39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1318,6 +1459,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr"/>
+      <c r="G40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1340,6 +1484,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E41" s="2" t="inlineStr"/>
+      <c r="F41" s="2" t="inlineStr"/>
+      <c r="G41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1362,6 +1509,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr"/>
+      <c r="G42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1384,6 +1534,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E43" s="2" t="inlineStr"/>
+      <c r="F43" s="2" t="inlineStr"/>
+      <c r="G43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1406,6 +1559,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1428,6 +1584,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E45" s="2" t="inlineStr"/>
+      <c r="F45" s="2" t="inlineStr"/>
+      <c r="G45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1450,6 +1609,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr"/>
+      <c r="G46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1472,6 +1634,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E47" s="2" t="inlineStr"/>
+      <c r="F47" s="2" t="inlineStr"/>
+      <c r="G47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1494,6 +1659,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr"/>
+      <c r="G48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -1516,6 +1684,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E49" s="2" t="inlineStr"/>
+      <c r="F49" s="2" t="inlineStr"/>
+      <c r="G49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1538,6 +1709,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr"/>
+      <c r="G50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -1560,6 +1734,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E51" s="2" t="inlineStr"/>
+      <c r="F51" s="2" t="inlineStr"/>
+      <c r="G51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -1582,6 +1759,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="inlineStr"/>
+      <c r="G52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -1604,6 +1784,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E53" s="2" t="inlineStr"/>
+      <c r="F53" s="2" t="inlineStr"/>
+      <c r="G53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -1626,6 +1809,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E54" s="2" t="inlineStr"/>
+      <c r="F54" s="2" t="inlineStr"/>
+      <c r="G54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -1648,6 +1834,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E55" s="2" t="inlineStr"/>
+      <c r="F55" s="2" t="inlineStr"/>
+      <c r="G55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -1670,6 +1859,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="inlineStr"/>
+      <c r="G56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -1692,6 +1884,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E57" s="2" t="inlineStr"/>
+      <c r="F57" s="2" t="inlineStr"/>
+      <c r="G57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -1714,6 +1909,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E58" s="2" t="inlineStr"/>
+      <c r="F58" s="2" t="inlineStr"/>
+      <c r="G58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -1736,6 +1934,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E59" s="2" t="inlineStr"/>
+      <c r="F59" s="2" t="inlineStr"/>
+      <c r="G59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -1758,6 +1959,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E60" s="2" t="inlineStr"/>
+      <c r="F60" s="2" t="inlineStr"/>
+      <c r="G60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -1780,6 +1984,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E61" s="2" t="inlineStr"/>
+      <c r="F61" s="2" t="inlineStr"/>
+      <c r="G61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -1802,6 +2009,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E62" s="2" t="inlineStr"/>
+      <c r="F62" s="2" t="inlineStr"/>
+      <c r="G62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -1824,6 +2034,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E63" s="2" t="inlineStr"/>
+      <c r="F63" s="2" t="inlineStr"/>
+      <c r="G63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -1846,6 +2059,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E64" s="2" t="inlineStr"/>
+      <c r="F64" s="2" t="inlineStr"/>
+      <c r="G64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -1868,6 +2084,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E65" s="2" t="inlineStr"/>
+      <c r="F65" s="2" t="inlineStr"/>
+      <c r="G65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -1890,6 +2109,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E66" s="2" t="inlineStr"/>
+      <c r="F66" s="2" t="inlineStr"/>
+      <c r="G66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -1912,6 +2134,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E67" s="2" t="inlineStr"/>
+      <c r="F67" s="2" t="inlineStr"/>
+      <c r="G67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -1934,6 +2159,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E68" s="2" t="inlineStr"/>
+      <c r="F68" s="2" t="inlineStr"/>
+      <c r="G68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -1956,6 +2184,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E69" s="2" t="inlineStr"/>
+      <c r="F69" s="2" t="inlineStr"/>
+      <c r="G69" s="2" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -1978,6 +2209,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E70" s="2" t="inlineStr"/>
+      <c r="F70" s="2" t="inlineStr"/>
+      <c r="G70" s="2" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -2000,6 +2234,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E71" s="2" t="inlineStr"/>
+      <c r="F71" s="2" t="inlineStr"/>
+      <c r="G71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -2022,6 +2259,9 @@
           <t>Autommerce OS</t>
         </is>
       </c>
+      <c r="E72" s="2" t="inlineStr"/>
+      <c r="F72" s="2" t="inlineStr"/>
+      <c r="G72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -2044,6 +2284,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E73" s="2" t="inlineStr"/>
+      <c r="F73" s="2" t="inlineStr"/>
+      <c r="G73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -2066,6 +2309,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E74" s="2" t="inlineStr"/>
+      <c r="F74" s="2" t="inlineStr"/>
+      <c r="G74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -2088,6 +2334,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E75" s="2" t="inlineStr"/>
+      <c r="F75" s="2" t="inlineStr"/>
+      <c r="G75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -2110,6 +2359,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E76" s="2" t="inlineStr"/>
+      <c r="F76" s="2" t="inlineStr"/>
+      <c r="G76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -2132,6 +2384,9 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E77" s="2" t="inlineStr"/>
+      <c r="F77" s="2" t="inlineStr"/>
+      <c r="G77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -2154,9 +2409,76 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="E78" s="2" t="inlineStr"/>
+      <c r="F78" s="2" t="inlineStr"/>
+      <c r="G78" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D78"/>
+  <autoFilter ref="A1:G78"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="001F4E79"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Decision Maker Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Company Name</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>